<commit_message>
docs: add more verified quantum graph papers
</commit_message>
<xml_diff>
--- a/metadata/QGraph.xlsx
+++ b/metadata/QGraph.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7f04913df7e94de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra06d23083b2a4fc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,388 +419,388 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
+        <x:v>Permutation-Invariant Quantum Graph Neural Network Based on Variational Quantum Algorithms</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Maoduo Li; Wen Liu; Lei Shi; Yangzhi Li; Weiping Ding</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>https://doi.org/10.1109/TNNLS.2026.3709916</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Feature prediction in quantum graph recurrent neural networks with applications in information hiding</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Springer Nature</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Jawaher Kaldari; Saif Al-Kuwari</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>https://doi.org/10.1007/s11128-026-05069-5</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Representational efficiency and noise robustness in hybrid quantum-classical graph neural networks</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Springer Nature</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Istiyak Amin Santo; Hasanul Bannah; Md Serajun Nabi et al.</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>https://doi.org/10.1007/s44464-026-00025-9</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Single-qubit graph classifier with classical feature aggregation</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Shaochun Li; Junzhi Cui; Jingli Ren</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>https://doi.org/10.1016/j.neunet.2026.108775</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>A Laplacian-based quantum graph neural networks for quantum semi-supervised learning</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Springer Nature</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Hamed Gholipour; Farid Bozorgnia; Kailash Hambarde; Hamzeh Mohammadigheymasi; Javier Mancilla; Andre Sequeira; João Neves; Hugo Proença; Moharram Challenger</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>https://doi.org/10.1007/s11128-025-04725-6</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
         <x:v>Quantum graphs: Different perspectives, homomorphisms and quantum automorphisms
 </x:v>
       </x:c>
-      <x:c r="B6" t="n">
+      <x:c r="B11" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C6" t="str">
+      <x:c r="C11" t="str">
         <x:v>Communications of the American Mathematical Society</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D11" t="str">
         <x:v>Daws, Matthew.</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E11" t="str">
         <x:v>https://www.ams.org/journals/cams/2024-04-05/S2692-3688-2024-00030-5/</x:v>
       </x:c>
-      <x:c r="F6" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="F11" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
         <x:v>Algebraic Connectedness and Bipartiteness of Quantum Graphs</x:v>
       </x:c>
-      <x:c r="B7" t="n">
+      <x:c r="B12" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C7" t="str">
+      <x:c r="C12" t="str">
         <x:v>Communications in Mathematical Physics</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D12" t="str">
         <x:v>Matsuda, Junichiro.</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E12" t="str">
         <x:v>https://link.springer.com/article/10.1007/s00220-024-05046-y</x:v>
       </x:c>
-      <x:c r="F7" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="F12" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
         <x:v>Financial fraud detection using quantum graph neural networks</x:v>
       </x:c>
-      <x:c r="B8" t="n">
+      <x:c r="B13" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C8" t="str">
+      <x:c r="C13" t="str">
         <x:v>Quantum Machine Intelligence </x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D13" t="str">
         <x:v>Innan, Nouhaila, et al.</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="E13" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42484-024-00143-6</x:v>
       </x:c>
-      <x:c r="F8" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="F13" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
         <x:v>A Comparison between Invariant and Equivariant Classical and Quantum Graph Neural Networks
 </x:v>
       </x:c>
-      <x:c r="B9" t="n">
+      <x:c r="B14" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C9" t="str">
+      <x:c r="C14" t="str">
         <x:v>Axioms</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D14" t="str">
         <x:v>Forestano, Roy T., et al.</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="E14" t="str">
         <x:v>https://www.mdpi.com/2075-1680/13/3/160</x:v>
       </x:c>
-      <x:c r="F9" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="F14" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
         <x:v>Deep quantum graph dreaming: deciphering neural network insights into quantum experiments
 </x:v>
       </x:c>
-      <x:c r="B10" t="n">
+      <x:c r="B15" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C15" t="str">
         <x:v>Machine Learning: Science and Technology</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D15" t="str">
         <x:v>Jaouni, Tareq, et al.</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E15" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ad2628/meta</x:v>
       </x:c>
-      <x:c r="F10" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="F15" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
         <x:v>Time evolution and the Schrödinger equation on
 time dependent quantum graphs</x:v>
       </x:c>
-      <x:c r="B11" t="n">
+      <x:c r="B16" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C16" t="str">
         <x:v>Journal of Physics A: Mathematical and Theoretical</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D16" t="str">
         <x:v>Smilansky, Uzy, and Gilad Sofer.</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E16" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/1751-8121/ad1fb6/meta</x:v>
       </x:c>
-      <x:c r="F11" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
+      <x:c r="F16" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
         <x:v>Invariants of the quantum graph of the partial trace
 </x:v>
       </x:c>
-      <x:c r="B12" t="n">
+      <x:c r="B17" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C12" t="str">
+      <x:c r="C17" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D17" t="str">
         <x:v>Paupa, Wojciech, and Piotr M. Sołtan.</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E17" t="str">
         <x:v>https://arxiv.org/abs/2408.16858</x:v>
       </x:c>
-      <x:c r="F12" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+      <x:c r="F17" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
         <x:v>QBER: Quantum-based Entropic Representations for un-attributed graphs</x:v>
       </x:c>
-      <x:c r="B13" t="n">
+      <x:c r="B18" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C18" t="str">
         <x:v>Pattern Recognition 1</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D18" t="str">
         <x:v>Cui, Lixin, et al.</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E18" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0031320323005757</x:v>
       </x:c>
-      <x:c r="F13" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
+      <x:c r="F18" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
         <x:v>Quantum isomorphism of graphs from association schemes</x:v>
       </x:c>
-      <x:c r="B14" t="n">
+      <x:c r="B19" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C19" t="str">
         <x:v>Journal of Combinatorial Theory</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D19" t="str">
         <x:v>Chan, Ada, and William J. Martin.</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E19" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0095895623000813</x:v>
       </x:c>
-      <x:c r="F14" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+      <x:c r="F19" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
         <x:v>HAQJSK: Hierarchical-Aligned Quantum Jensen-Shannon Kernels for Graph Classification
 </x:v>
       </x:c>
-      <x:c r="B15" t="n">
+      <x:c r="B20" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C15" t="str">
+      <x:c r="C20" t="str">
         <x:v>IEEE Transactions on Knowledge and Data Engineering</x:v>
       </x:c>
-      <x:c r="D15" t="str">
+      <x:c r="D20" t="str">
         <x:v>Bai, Lu, et al.</x:v>
       </x:c>
-      <x:c r="E15" t="str">
+      <x:c r="E20" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10502132</x:v>
       </x:c>
-      <x:c r="F15" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
+      <x:c r="F20" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
         <x:v>A Quantum Spatial Graph Convolutional Neural Network Model on Quantum Circuits
 </x:v>
       </x:c>
-      <x:c r="B16" t="n">
+      <x:c r="B21" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C21" t="str">
         <x:v>IEEE Transactions on Neural Networks and Learning Systems </x:v>
       </x:c>
-      <x:c r="D16" t="str">
+      <x:c r="D21" t="str">
         <x:v>Zheng, Jin, et al.</x:v>
       </x:c>
-      <x:c r="E16" t="str">
+      <x:c r="E21" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10499715</x:v>
       </x:c>
-      <x:c r="F16" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
+      <x:c r="F21" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
         <x:v>Quantum Feature Embeddings for Graph Neural Networks</x:v>
       </x:c>
-      <x:c r="B17" t="n">
+      <x:c r="B22" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C17" t="str">
+      <x:c r="C22" t="str">
         <x:v>HICSS</x:v>
       </x:c>
-      <x:c r="D17" t="str">
+      <x:c r="D22" t="str">
         <x:v>Xu, Sascha, Frank Wilhelm-Mauch, and Wolfgang Maass.</x:v>
       </x:c>
-      <x:c r="E17" t="str">
+      <x:c r="E22" t="str">
         <x:v>https://www.quasim-project.de/wp-content/uploads/2023/09/Quantum-Feature-Embeddings-for-Graph-Neural-Networks_HICSS2024.pdf</x:v>
       </x:c>
-      <x:c r="F17" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
+      <x:c r="F22" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
         <x:v>Quantum Positional Encodings for Graph Neural Networks
 </x:v>
       </x:c>
-      <x:c r="B18" t="n">
+      <x:c r="B23" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C18" t="str">
+      <x:c r="C23" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D18" t="str">
+      <x:c r="D23" t="str">
         <x:v>Thabet, Slimane, et al.</x:v>
       </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="E23" t="str">
         <x:v>https://arxiv.org/abs/2406.06547</x:v>
       </x:c>
-      <x:c r="F18" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
+      <x:c r="F23" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
         <x:v>GraphiQ: Quantum circuit design for photonic graph states
 </x:v>
       </x:c>
-      <x:c r="B19" t="n">
+      <x:c r="B24" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C19" t="str">
+      <x:c r="C24" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D19" t="str">
+      <x:c r="D24" t="str">
         <x:v>Lin, Jie, et al.</x:v>
       </x:c>
-      <x:c r="E19" t="str">
+      <x:c r="E24" t="str">
         <x:v>https://arxiv.org/abs/2402.09285</x:v>
-      </x:c>
-      <x:c r="F19" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>Interaction graph-based characterization of quantum benchmarks for improving quantum circuit mapping techniques</x:v>
-      </x:c>
-      <x:c r="B20" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>Medina Bandic, Carmen G. Almudever, Sebastian Feld </x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00124-1</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>Very-large-scale integrated quantum graph photonics</x:v>
-      </x:c>
-      <x:c r="B21" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C21" t="str">
-        <x:v>Nature Photonics</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>Jueming Bao, Zhaorong Fu, Tanumoy Pramanik, Jun Mao, Yulin Chi, Yingkang Cao, Chonghao Zhai, Yifei Mao, Tianxiang Dai, Xiaojiong Chen, Xinyu Jia, Leshi Zhao, Yun Zheng, Bo Tang, Zhihua Li, Jun Luo, Wenwu Wang, Yan Yang, Yingying Peng, Dajian Liu, Daoxin Dai, Qiongyi He, Alif Laila Muthali, Leif K. Oxenløwe, Caterina Vigliar, Stefano Paesani, Huili Hou, Raffaele Santagati, Joshua W. Silverstone, Anthony Laing, Mark G. Thompson, Jeremy L. O’Brien, Yunhong Ding, Qihuang Gong &amp; Jianwei Wang</x:v>
-      </x:c>
-      <x:c r="E21" t="str">
-        <x:v>https://doi.org/10.1038/s41566-023-01187-z</x:v>
-      </x:c>
-      <x:c r="F21" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" t="str">
-        <x:v>GCS-Q: Quantum Graph Coalition Structure Generation</x:v>
-      </x:c>
-      <x:c r="B22" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C22" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D22" t="str">
-        <x:v>Supreeth Mysore Venkatesh, Antonio Macaluso &amp; Matthias Klusch </x:v>
-      </x:c>
-      <x:c r="E22" t="str">
-        <x:v>https://doi.org/10.1007/978-3-031-36030-5_11</x:v>
-      </x:c>
-      <x:c r="F22" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" t="str">
-        <x:v>Deep learning metal complex properties with natural quantum graphs</x:v>
-      </x:c>
-      <x:c r="B23" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C23" t="str">
-        <x:v>ROYAL SOCIETY OF CHEMISTRY</x:v>
-      </x:c>
-      <x:c r="D23" t="str">
-        <x:v>Hannes Kneiding, Ruslan Lukin a, Lucas Lang , Simen Reine logoa, Thomas Bondo Pedersen, Riccardo De Bin , David Balcells</x:v>
-      </x:c>
-      <x:c r="E23" t="str">
-        <x:v>https://doi.org/10.1039/D2DD00129B</x:v>
-      </x:c>
-      <x:c r="F23" t="str">
-        <x:v>Qgraph</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="str">
-        <x:v>Distinguishing cospectral quantum graphs by scattering</x:v>
-      </x:c>
-      <x:c r="B24" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C24" t="str">
-        <x:v>IOPSCIENCE</x:v>
-      </x:c>
-      <x:c r="D24" t="str">
-        <x:v>Delio Mugnolo and Vyacheslav Pivovarchik</x:v>
-      </x:c>
-      <x:c r="E24" t="str">
-        <x:v>https://doi.org/10.1088/1751-8121/acbb44</x:v>
       </x:c>
       <x:c r="F24" t="str">
         <x:v>Qgraph</x:v>
@@ -808,19 +808,19 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>Equivariant quantum circuits for learning on weighted graphs</x:v>
+        <x:v>Interaction graph-based characterization of quantum benchmarks for improving quantum circuit mapping techniques</x:v>
       </x:c>
       <x:c r="B25" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>npj Quantum Information</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>Andrea Skolik, Michele Cattelan, Sheir Yarkoni, Thomas Bäck &amp; Vedran Dunjko</x:v>
+        <x:v>Medina Bandic, Carmen G. Almudever, Sebastian Feld </x:v>
       </x:c>
       <x:c r="E25" t="str">
-        <x:v>https://doi.org/10.1038/s41534-023-00710-y</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00124-1</x:v>
       </x:c>
       <x:c r="F25" t="str">
         <x:v>Qgraph</x:v>
@@ -828,19 +828,19 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
-        <x:v>Quantum feature maps for graph machine learning on a neutral atom quantum processor</x:v>
+        <x:v>Very-large-scale integrated quantum graph photonics</x:v>
       </x:c>
       <x:c r="B26" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>APS</x:v>
+        <x:v>Nature Photonics</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>Boris Albrecht, Constantin Dalyac, Lucas Leclerc, Luis Ortiz-Gutiérrez, Slimane Thabet, Mauro D'Arcangelo, Julia R. K. Cline, Vincent E. Elfving, Lucas Lassablière, Henrique Silvério, Bruno Ximenez, Louis-Paul Henry, Adrien Signoles, and Loïc Henriet</x:v>
+        <x:v>Jueming Bao, Zhaorong Fu, Tanumoy Pramanik, Jun Mao, Yulin Chi, Yingkang Cao, Chonghao Zhai, Yifei Mao, Tianxiang Dai, Xiaojiong Chen, Xinyu Jia, Leshi Zhao, Yun Zheng, Bo Tang, Zhihua Li, Jun Luo, Wenwu Wang, Yan Yang, Yingying Peng, Dajian Liu, Daoxin Dai, Qiongyi He, Alif Laila Muthali, Leif K. Oxenløwe, Caterina Vigliar, Stefano Paesani, Huili Hou, Raffaele Santagati, Joshua W. Silverstone, Anthony Laing, Mark G. Thompson, Jeremy L. O’Brien, Yunhong Ding, Qihuang Gong &amp; Jianwei Wang</x:v>
       </x:c>
       <x:c r="E26" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevA.107.042615</x:v>
+        <x:v>https://doi.org/10.1038/s41566-023-01187-z</x:v>
       </x:c>
       <x:c r="F26" t="str">
         <x:v>Qgraph</x:v>
@@ -848,19 +848,19 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>Advantages and Limitations of Quantum Routing</x:v>
+        <x:v>GCS-Q: Quantum Graph Coalition Structure Generation</x:v>
       </x:c>
       <x:c r="B27" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>APS</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D27" t="str">
-        <x:v>Aniruddha Bapat, Andrew M. Childs, Alexey V. Gorshkov, and Eddie Schoute</x:v>
+        <x:v>Supreeth Mysore Venkatesh, Antonio Macaluso &amp; Matthias Klusch </x:v>
       </x:c>
       <x:c r="E27" t="str">
-        <x:v>https://doi.org/10.1103/PRXQuantum.4.010313</x:v>
+        <x:v>https://doi.org/10.1007/978-3-031-36030-5_11</x:v>
       </x:c>
       <x:c r="F27" t="str">
         <x:v>Qgraph</x:v>
@@ -868,19 +868,19 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>Method for solving inverse spectral problems on quantum star graphs</x:v>
+        <x:v>Deep learning metal complex properties with natural quantum graphs</x:v>
       </x:c>
       <x:c r="B28" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>DE GRUYTER</x:v>
+        <x:v>ROYAL SOCIETY OF CHEMISTRY</x:v>
       </x:c>
       <x:c r="D28" t="str">
-        <x:v>Sergei A. Avdonin and Vladislav V. Kravchenko</x:v>
+        <x:v>Hannes Kneiding, Ruslan Lukin a, Lucas Lang , Simen Reine logoa, Thomas Bondo Pedersen, Riccardo De Bin , David Balcells</x:v>
       </x:c>
       <x:c r="E28" t="str">
-        <x:v>https://doi.org/10.1515/jiip-2022-0045</x:v>
+        <x:v>https://doi.org/10.1039/D2DD00129B</x:v>
       </x:c>
       <x:c r="F28" t="str">
         <x:v>Qgraph</x:v>
@@ -888,19 +888,19 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
-        <x:v>Graph-theoretical optimization of fusion-based graph state generation</x:v>
+        <x:v>Distinguishing cospectral quantum graphs by scattering</x:v>
       </x:c>
       <x:c r="B29" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>the open journal for quantum science</x:v>
+        <x:v>IOPSCIENCE</x:v>
       </x:c>
       <x:c r="D29" t="str">
-        <x:v>Seok-Hyung Lee, Hyunseok Jeong</x:v>
+        <x:v>Delio Mugnolo and Vyacheslav Pivovarchik</x:v>
       </x:c>
       <x:c r="E29" t="str">
-        <x:v>https://doi.org/10.22331/q-2023-12-20-1212</x:v>
+        <x:v>https://doi.org/10.1088/1751-8121/acbb44</x:v>
       </x:c>
       <x:c r="F29" t="str">
         <x:v>Qgraph</x:v>
@@ -908,19 +908,19 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>Quantum Automorphism Groups of Connected Locally Finite Graphs and Quantizations of Discrete Groups</x:v>
+        <x:v>Equivariant quantum circuits for learning on weighted graphs</x:v>
       </x:c>
       <x:c r="B30" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>Journal of the American Mathematical Society</x:v>
+        <x:v>npj Quantum Information</x:v>
       </x:c>
       <x:c r="D30" t="str">
-        <x:v>Lukas Rollier, Stefaan Vaes</x:v>
+        <x:v>Andrea Skolik, Michele Cattelan, Sheir Yarkoni, Thomas Bäck &amp; Vedran Dunjko</x:v>
       </x:c>
       <x:c r="E30" t="str">
-        <x:v>https://doi.org/10.1093/imrn/rnad099</x:v>
+        <x:v>https://doi.org/10.1038/s41534-023-00710-y</x:v>
       </x:c>
       <x:c r="F30" t="str">
         <x:v>Qgraph</x:v>
@@ -928,19 +928,19 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
-        <x:v>GSQAS: Graph Self-supervised Quantum Architecture Search</x:v>
+        <x:v>Quantum feature maps for graph machine learning on a neutral atom quantum processor</x:v>
       </x:c>
       <x:c r="B31" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>APS</x:v>
       </x:c>
       <x:c r="D31" t="str">
-        <x:v>Zhimin He, Maijie Deng, Shenggen Zheng, Lvzhou Li, Haozhen Situ</x:v>
+        <x:v>Boris Albrecht, Constantin Dalyac, Lucas Leclerc, Luis Ortiz-Gutiérrez, Slimane Thabet, Mauro D'Arcangelo, Julia R. K. Cline, Vincent E. Elfving, Lucas Lassablière, Henrique Silvério, Bruno Ximenez, Louis-Paul Henry, Adrien Signoles, and Loïc Henriet</x:v>
       </x:c>
       <x:c r="E31" t="str">
-        <x:v>https://doi.org/10.1016/j.physa.2023.129286</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevA.107.042615</x:v>
       </x:c>
       <x:c r="F31" t="str">
         <x:v>Qgraph</x:v>
@@ -948,19 +948,19 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
-        <x:v>On the Design of Quantum Graph Convolutional Neural Network in the NISQ-Era and Beyond</x:v>
+        <x:v>Advantages and Limitations of Quantum Routing</x:v>
       </x:c>
       <x:c r="B32" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>IEEE International Conference on Computer Design: VLSI in Computers and Processors, (ICCD)</x:v>
+        <x:v>APS</x:v>
       </x:c>
       <x:c r="D32" t="str">
-        <x:v>Zhirui Hu; Jinyang Li; Zhenyu Pan; Shanglin Zhou; Lei Yang; Caiwen Ding</x:v>
+        <x:v>Aniruddha Bapat, Andrew M. Childs, Alexey V. Gorshkov, and Eddie Schoute</x:v>
       </x:c>
       <x:c r="E32" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9978396</x:v>
+        <x:v>https://doi.org/10.1103/PRXQuantum.4.010313</x:v>
       </x:c>
       <x:c r="F32" t="str">
         <x:v>Qgraph</x:v>
@@ -968,19 +968,19 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>Data-Driven Reliability Models of Quantum Circuit: From Traditional ML to Graph Neural Network</x:v>
+        <x:v>Method for solving inverse spectral problems on quantum star graphs</x:v>
       </x:c>
       <x:c r="B33" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>IEEE Transactions on Computer-Aided Design of Integrated Circuits and Systems</x:v>
+        <x:v>DE GRUYTER</x:v>
       </x:c>
       <x:c r="D33" t="str">
-        <x:v>Vedika Saravanan; Samah M. Saeed</x:v>
+        <x:v>Sergei A. Avdonin and Vladislav V. Kravchenko</x:v>
       </x:c>
       <x:c r="E33" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9877896</x:v>
+        <x:v>https://doi.org/10.1515/jiip-2022-0045</x:v>
       </x:c>
       <x:c r="F33" t="str">
         <x:v>Qgraph</x:v>
@@ -988,19 +988,19 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>Equivariant Quantum Graph Circuits</x:v>
+        <x:v>Graph-theoretical optimization of fusion-based graph state generation</x:v>
       </x:c>
       <x:c r="B34" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>International Conference on Machine Learning</x:v>
+        <x:v>the open journal for quantum science</x:v>
       </x:c>
       <x:c r="D34" t="str">
-        <x:v>Peter Mernyei, Konstantinos Meichanetzidis, Ismail Ilkan Ceylan</x:v>
+        <x:v>Seok-Hyung Lee, Hyunseok Jeong</x:v>
       </x:c>
       <x:c r="E34" t="str">
-        <x:v>https://proceedings.mlr.press/v162/mernyei22a.html</x:v>
+        <x:v>https://doi.org/10.22331/q-2023-12-20-1212</x:v>
       </x:c>
       <x:c r="F34" t="str">
         <x:v>Qgraph</x:v>
@@ -1008,19 +1008,19 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>A quantum graph approach to metamaterial design</x:v>
+        <x:v>Quantum Automorphism Groups of Connected Locally Finite Graphs and Quantizations of Discrete Groups</x:v>
       </x:c>
       <x:c r="B35" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>Scientific Reports</x:v>
+        <x:v>Journal of the American Mathematical Society</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>      Tristan Lawrie, Gregor Tanner &amp; Dimitrios Chronopoulos   </x:v>
+        <x:v>Lukas Rollier, Stefaan Vaes</x:v>
       </x:c>
       <x:c r="E35" t="str">
-        <x:v>https://www.nature.com/articles/s41598-022-22265-2</x:v>
+        <x:v>https://doi.org/10.1093/imrn/rnad099</x:v>
       </x:c>
       <x:c r="F35" t="str">
         <x:v>Qgraph</x:v>
@@ -1028,19 +1028,19 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
-        <x:v>Temporal-Spatial Quantum Graph Convolutional Neural Network Based on Schrödinger Approach for Traffic Congestion Prediction</x:v>
+        <x:v>GSQAS: Graph Self-supervised Quantum Architecture Search</x:v>
       </x:c>
       <x:c r="B36" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>IEEE Transactions on Intelligent Transportation Systems</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D36" t="str">
-        <x:v>Zhiguo Qu; Xinzhu Liu; Min Zheng</x:v>
+        <x:v>Zhimin He, Maijie Deng, Shenggen Zheng, Lvzhou Li, Haozhen Situ</x:v>
       </x:c>
       <x:c r="E36" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9882032</x:v>
+        <x:v>https://doi.org/10.1016/j.physa.2023.129286</x:v>
       </x:c>
       <x:c r="F36" t="str">
         <x:v>Qgraph</x:v>
@@ -1048,19 +1048,19 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
-        <x:v>Towards Quantum Graph Neural Networks: An Ego-Graph Learning Approach</x:v>
+        <x:v>On the Design of Quantum Graph Convolutional Neural Network in the NISQ-Era and Beyond</x:v>
       </x:c>
       <x:c r="B37" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>inspirehep</x:v>
+        <x:v>IEEE International Conference on Computer Design: VLSI in Computers and Processors, (ICCD)</x:v>
       </x:c>
       <x:c r="D37" t="str">
-        <x:v>Xing Ai(      Xiamen U.  ) , Zhihong Zhang(      Xiamen U.  ) , Luzhe Sun(      Xiamen U.  ) , Junchi Yan(      Shanghai Jiao Tong U.  ) , Edwin Hancock</x:v>
+        <x:v>Zhirui Hu; Jinyang Li; Zhenyu Pan; Shanglin Zhou; Lei Yang; Caiwen Ding</x:v>
       </x:c>
       <x:c r="E37" t="str">
-        <x:v>https://inspirehep.net/literature/2011088</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9978396</x:v>
       </x:c>
       <x:c r="F37" t="str">
         <x:v>Qgraph</x:v>
@@ -1068,19 +1068,19 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>Random quantum graphs</x:v>
+        <x:v>Data-Driven Reliability Models of Quantum Circuit: From Traditional ML to Graph Neural Network</x:v>
       </x:c>
       <x:c r="B38" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>Trans. Amer. Math. Soc. 375 (2022)</x:v>
+        <x:v>IEEE Transactions on Computer-Aided Design of Integrated Circuits and Systems</x:v>
       </x:c>
       <x:c r="D38" t="str">
-        <x:v>Alexandru Chirvasitu and Mateusz Wasilewski</x:v>
+        <x:v>Vedika Saravanan; Samah M. Saeed</x:v>
       </x:c>
       <x:c r="E38" t="str">
-        <x:v>https://www.ams.org/journals/tran/2022-375-05/S0002-9947-2022-08584-6/home.html</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9877896</x:v>
       </x:c>
       <x:c r="F38" t="str">
         <x:v>Qgraph</x:v>
@@ -1088,19 +1088,19 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
-        <x:v>Some examples of quantum graphs</x:v>
+        <x:v>Equivariant Quantum Graph Circuits</x:v>
       </x:c>
       <x:c r="B39" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>Letters in Mathematical Physics</x:v>
+        <x:v>International Conference on Machine Learning</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>Daniel Gromada </x:v>
+        <x:v>Peter Mernyei, Konstantinos Meichanetzidis, Ismail Ilkan Ceylan</x:v>
       </x:c>
       <x:c r="E39" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11005-022-01603-5</x:v>
+        <x:v>https://proceedings.mlr.press/v162/mernyei22a.html</x:v>
       </x:c>
       <x:c r="F39" t="str">
         <x:v>Qgraph</x:v>
@@ -1108,19 +1108,19 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
-        <x:v>Quantum-Chemical and Quantum-Graph Models of the Dynamical Structure of CH5+</x:v>
+        <x:v>A quantum graph approach to metamaterial design</x:v>
       </x:c>
       <x:c r="B40" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>Journal of Chemical Theory and Computation</x:v>
+        <x:v>Scientific Reports</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>Irén Simkó, Csaba Fábri, Attila G. Császár*</x:v>
+        <x:v>      Tristan Lawrie, Gregor Tanner &amp; Dimitrios Chronopoulos   </x:v>
       </x:c>
       <x:c r="E40" t="str">
-        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.jctc.2c00991</x:v>
+        <x:v>https://www.nature.com/articles/s41598-022-22265-2</x:v>
       </x:c>
       <x:c r="F40" t="str">
         <x:v>Qgraph</x:v>
@@ -1128,19 +1128,19 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
-        <x:v>From Quantum Graph Computing to Quantum Graph Learning: A Survey</x:v>
+        <x:v>Temporal-Spatial Quantum Graph Convolutional Neural Network Based on Schrödinger Approach for Traffic Congestion Prediction</x:v>
       </x:c>
       <x:c r="B41" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>IEEE Transactions on Intelligent Transportation Systems</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>Yehui Tang, Junchi Yan, Hancock Edwin</x:v>
+        <x:v>Zhiguo Qu; Xinzhu Liu; Min Zheng</x:v>
       </x:c>
       <x:c r="E41" t="str">
-        <x:v>https://arxiv.org/abs/2202.09506</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9882032</x:v>
       </x:c>
       <x:c r="F41" t="str">
         <x:v>Qgraph</x:v>
@@ -1148,19 +1148,19 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="str">
-        <x:v>Supervised graph classification for chiral quantum walks</x:v>
+        <x:v>Towards Quantum Graph Neural Networks: An Ego-Graph Learning Approach</x:v>
       </x:c>
       <x:c r="B42" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>Phys. Rev. A 105</x:v>
+        <x:v>inspirehep</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>Artem Kryukov, Roman Abramov, Leonid E. Fedichkin, Alexander Alodjants, and Alexey A. Melnikov</x:v>
+        <x:v>Xing Ai(      Xiamen U.  ) , Zhihong Zhang(      Xiamen U.  ) , Luzhe Sun(      Xiamen U.  ) , Junchi Yan(      Shanghai Jiao Tong U.  ) , Edwin Hancock</x:v>
       </x:c>
       <x:c r="E42" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.022208</x:v>
+        <x:v>https://inspirehep.net/literature/2011088</x:v>
       </x:c>
       <x:c r="F42" t="str">
         <x:v>Qgraph</x:v>
@@ -1168,19 +1168,19 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="str">
-        <x:v>Learning quantum graph states with product measurements</x:v>
+        <x:v>Random quantum graphs</x:v>
       </x:c>
       <x:c r="B43" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>2022 IEEE International Symposium on Information Theory (ISIT)</x:v>
+        <x:v>Trans. Amer. Math. Soc. 375 (2022)</x:v>
       </x:c>
       <x:c r="D43" t="str">
-        <x:v>Yingkai Ouyang; Marco Tomamichel</x:v>
+        <x:v>Alexandru Chirvasitu and Mateusz Wasilewski</x:v>
       </x:c>
       <x:c r="E43" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9834440</x:v>
+        <x:v>https://www.ams.org/journals/tran/2022-375-05/S0002-9947-2022-08584-6/home.html</x:v>
       </x:c>
       <x:c r="F43" t="str">
         <x:v>Qgraph</x:v>
@@ -1188,19 +1188,19 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="str">
-        <x:v>Quantum Mechanics and Machine Learning Synergies: Graph Attention Neural Networks to Predict Chemical Reactivity</x:v>
+        <x:v>Some examples of quantum graphs</x:v>
       </x:c>
       <x:c r="B44" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>Machine Learning and Deep Learning</x:v>
+        <x:v>Letters in Mathematical Physics</x:v>
       </x:c>
       <x:c r="D44" t="str">
-        <x:v>Mohammadamin TavakoliAaron MoodDavid Van VrankenPierre Baldi</x:v>
+        <x:v>Daniel Gromada </x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.jcim.1c01400</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11005-022-01603-5</x:v>
       </x:c>
       <x:c r="F44" t="str">
         <x:v>Qgraph</x:v>
@@ -1208,19 +1208,19 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="str">
-        <x:v>QuEst: Graph Transformer for Quantum Circuit Reliability Estimation</x:v>
+        <x:v>Quantum-Chemical and Quantum-Graph Models of the Dynamical Structure of CH5+</x:v>
       </x:c>
       <x:c r="B45" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Journal of Chemical Theory and Computation</x:v>
       </x:c>
       <x:c r="D45" t="str">
-        <x:v>Hanrui Wang, Pengyu Liu, Jinglei Cheng, Zhiding Liang, Jiaqi Gu, Zirui Li, Yongshan Ding, Weiwen Jiang, Yiyu Shi, Xuehai Qian, David Z. Pan, Frederic T. Chong, Song Han</x:v>
+        <x:v>Irén Simkó, Csaba Fábri, Attila G. Császár*</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>https://arxiv.org/abs/2210.16724</x:v>
+        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.jctc.2c00991</x:v>
       </x:c>
       <x:c r="F45" t="str">
         <x:v>Qgraph</x:v>
@@ -1228,7 +1228,7 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
-        <x:v>Novel Architecture of Parameterized Quantum Circuit for Graph Convolutional Network</x:v>
+        <x:v>From Quantum Graph Computing to Quantum Graph Learning: A Survey</x:v>
       </x:c>
       <x:c r="B46" t="n">
         <x:v>2022</x:v>
@@ -1237,10 +1237,10 @@
         <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D46" t="str">
-        <x:v>Yanhu Chen, Cen Wang, Hongxiang Guo, Jianwu</x:v>
+        <x:v>Yehui Tang, Junchi Yan, Hancock Edwin</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>https://arxiv.org/abs/2203.03251</x:v>
+        <x:v>https://arxiv.org/abs/2202.09506</x:v>
       </x:c>
       <x:c r="F46" t="str">
         <x:v>Qgraph</x:v>
@@ -1248,19 +1248,19 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
-        <x:v>Towards a Native Quantum Paradigm for Graph Representation Learning: A Sampling-based Recurrent Embedding Approach</x:v>
+        <x:v>Supervised graph classification for chiral quantum walks</x:v>
       </x:c>
       <x:c r="B47" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>KDD '22: Proceedings of the 28th ACM SIGKDD Conference on Knowledge Discovery and Data Mining</x:v>
+        <x:v>Phys. Rev. A 105</x:v>
       </x:c>
       <x:c r="D47" t="str">
-        <x:v>Ge Yan, Yehui Tang, Junchi Yan</x:v>
+        <x:v>Artem Kryukov, Roman Abramov, Leonid E. Fedichkin, Alexander Alodjants, and Alexey A. Melnikov</x:v>
       </x:c>
       <x:c r="E47" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3534678.3539327</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.022208</x:v>
       </x:c>
       <x:c r="F47" t="str">
         <x:v>Qgraph</x:v>
@@ -1268,19 +1268,19 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="str">
-        <x:v>QuanGCN: Noise-Adaptive Training for Robust Quantum Graph Convolutional Networks</x:v>
+        <x:v>Learning quantum graph states with product measurements</x:v>
       </x:c>
       <x:c r="B48" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>2022 IEEE International Symposium on Information Theory (ISIT)</x:v>
       </x:c>
       <x:c r="D48" t="str">
-        <x:v>Kaixiong Zhou, Zhenyu Zhang, Shengyuan Chen, Tianlong Chen, Xiao Huang, Zhangyang Wang, Xia Hu</x:v>
+        <x:v>Yingkai Ouyang; Marco Tomamichel</x:v>
       </x:c>
       <x:c r="E48" t="str">
-        <x:v>https://arxiv.org/abs/2211.07379</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9834440</x:v>
       </x:c>
       <x:c r="F48" t="str">
         <x:v>Qgraph</x:v>
@@ -1288,38 +1288,138 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" t="str">
+        <x:v>Quantum Mechanics and Machine Learning Synergies: Graph Attention Neural Networks to Predict Chemical Reactivity</x:v>
+      </x:c>
+      <x:c r="B49" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Machine Learning and Deep Learning</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Mohammadamin TavakoliAaron MoodDavid Van VrankenPierre Baldi</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.jcim.1c01400</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>QuEst: Graph Transformer for Quantum Circuit Reliability Estimation</x:v>
+      </x:c>
+      <x:c r="B50" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Hanrui Wang, Pengyu Liu, Jinglei Cheng, Zhiding Liang, Jiaqi Gu, Zirui Li, Yongshan Ding, Weiwen Jiang, Yiyu Shi, Xuehai Qian, David Z. Pan, Frederic T. Chong, Song Han</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>https://arxiv.org/abs/2210.16724</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>Novel Architecture of Parameterized Quantum Circuit for Graph Convolutional Network</x:v>
+      </x:c>
+      <x:c r="B51" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>Yanhu Chen, Cen Wang, Hongxiang Guo, Jianwu</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>https://arxiv.org/abs/2203.03251</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>Towards a Native Quantum Paradigm for Graph Representation Learning: A Sampling-based Recurrent Embedding Approach</x:v>
+      </x:c>
+      <x:c r="B52" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>KDD '22: Proceedings of the 28th ACM SIGKDD Conference on Knowledge Discovery and Data Mining</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>Ge Yan, Yehui Tang, Junchi Yan</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3534678.3539327</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>QuanGCN: Noise-Adaptive Training for Robust Quantum Graph Convolutional Networks</x:v>
+      </x:c>
+      <x:c r="B53" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Kaixiong Zhou, Zhenyu Zhang, Shengyuan Chen, Tianlong Chen, Xiao Huang, Zhangyang Wang, Xia Hu</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>https://arxiv.org/abs/2211.07379</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>Qgraph</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
         <x:v>Qubit Routing Using Graph Neural Network Aided Monte Carlo Tree Search</x:v>
       </x:c>
-      <x:c r="B49" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C49" t="str">
+      <x:c r="B54" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
         <x:v>AAAI Technical Track on Planning, Routing, and Scheduling </x:v>
       </x:c>
-      <x:c r="D49" t="str">
+      <x:c r="D54" t="str">
         <x:v>Animesh Sinha </x:v>
       </x:c>
-      <x:c r="E49" t="str">
+      <x:c r="E54" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/21231</x:v>
       </x:c>
-      <x:c r="F49" t="str">
+      <x:c r="F54" t="str">
         <x:v>Qgraph</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R3c5eb7f0da1b4db0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R22e247bb4bb84e93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Re251075bd9804ce0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R5d43cc3ceffd4227"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="Rf0a04119009f4834"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Rc52075685b6d4117"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Rd14bf3cf638b4fab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rea6b7d97d41d444d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R3b0394631caa4d8a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rb9804ffa18084ca7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R7764f90769e1484c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R93b617a449184eb4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R1e5fee228ee54021"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R696f0508172b4b38"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Rfd7689c80e4b4253"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="Rfd3fb8477c2f4927"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R6f9bbb9744644ccc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R10a1b0d19b7f4eea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Rd1453b66cef74c46"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R116753ecd67b49f2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R1d1b62819fcc48b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rf9a88cee413d4f86"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R250887d6a9274c59"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R9fb24bca89564f0a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>